<commit_message>
Locate internal electrical installations item in the acta
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G7N1VJagVFte3WPhVVEECp
</commit_message>
<xml_diff>
--- a/Revision_Electrica_IDER_Bayunca.xlsx
+++ b/Revision_Electrica_IDER_Bayunca.xlsx
@@ -7413,7 +7413,7 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>INSTALACIONES ELECTRICAS (INTERNAS)</t>
+          <t>INSTALACIONES ELECTRICAS (INTERNAS) [hoja ACTA MAY Y MEN, fila 349, bloque MÓDULO DE SERVICIO 7X14 (IN15), sin código]</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="Q88" s="4" t="inlineStr">
         <is>
-          <t>Global de $8,0 M: posible duplicidad con 4.30 a 4.38 e IN14.12 a IN14.17.</t>
+          <t>Ubicado en la hoja ACTA MAY Y MEN, fila 349, dentro del bloque MÓDULO DE SERVICIO 7X14 (IN15) y sin código. Global de $8,0 M: posible duplicidad con 4.30 a 4.38 e IN14.12 a IN14.17.</t>
         </is>
       </c>
       <c r="R88" s="4" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Ítem global que puede duplicar 4.30 a 4.38 e IN14.12 a IN14.17.</t>
+          <t>Ítem global sin código (hoja ACTA MAY Y MEN, fila 349, bloque MÓDULO DE SERVICIO 7X14) que puede duplicar 4.30 a 4.38 e IN14.12 a IN14.17.</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Make validated-quantity column blank for supervisor input
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G7N1VJagVFte3WPhVVEECp
</commit_message>
<xml_diff>
--- a/Revision_Electrica_IDER_Bayunca.xlsx
+++ b/Revision_Electrica_IDER_Bayunca.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items_Electricos'!$A$4:$W$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items_Electricos'!$A$4:$X$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Matriz_Observaciones'!$A$4:$R$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Formato_Blanco'!$A$4:$R$204</definedName>
   </definedNames>
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -332,6 +332,13 @@
     <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1708,21 +1715,21 @@
     <row r="61">
       <c r="A61" s="36" t="inlineStr">
         <is>
-          <t>Balance ajustado (ítems eléctricos)</t>
+          <t>Presupuesto validado (ítems eléctricos)</t>
         </is>
       </c>
       <c r="B61" s="37">
-        <f>Items_Electricos!U107</f>
+        <f>Items_Electricos!U106</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="36" t="inlineStr">
         <is>
-          <t>Pendiente de validar</t>
-        </is>
-      </c>
-      <c r="B62" s="37">
+          <t>Ítems pendientes de validar</t>
+        </is>
+      </c>
+      <c r="B62" s="56">
         <f>Items_Electricos!U109</f>
         <v/>
       </c>
@@ -1740,7 +1747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W111"/>
+  <dimension ref="A1:X112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1764,6 +1771,7 @@
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="50" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1878,7 +1886,7 @@
       </c>
       <c r="T4" s="38" t="inlineStr">
         <is>
-          <t>Cant. ajustada validada (supervisor)</t>
+          <t>Cant. validada por el supervisor (diligenciar)</t>
         </is>
       </c>
       <c r="U4" s="38" t="inlineStr">
@@ -1893,7 +1901,12 @@
       </c>
       <c r="W4" s="38" t="inlineStr">
         <is>
-          <t>Validación</t>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="X4" s="38" t="inlineStr">
+        <is>
+          <t>Observaciones del supervisor</t>
         </is>
       </c>
     </row>
@@ -1994,23 +2007,20 @@
           <t>OBS-021</t>
         </is>
       </c>
-      <c r="T6" s="42">
-        <f>I6</f>
-        <v/>
-      </c>
+      <c r="T6" s="42" t="n"/>
       <c r="U6" s="43">
-        <f>T6*N(F6)</f>
+        <f>IF(T6="",0,T6*N(F6))</f>
         <v/>
       </c>
       <c r="V6" s="43">
-        <f>U6-J6</f>
-        <v/>
-      </c>
-      <c r="W6" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T6="","",U6-J6)</f>
+        <v/>
+      </c>
+      <c r="W6" s="44">
+        <f>IF(T6="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X6" s="57" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="21" t="n"/>
@@ -2156,23 +2166,20 @@
           <t>OBS-039</t>
         </is>
       </c>
-      <c r="T9" s="42">
-        <f>I9</f>
-        <v/>
-      </c>
+      <c r="T9" s="42" t="n"/>
       <c r="U9" s="43">
-        <f>T9*N(F9)</f>
+        <f>IF(T9="",0,T9*N(F9))</f>
         <v/>
       </c>
       <c r="V9" s="43">
-        <f>U9-J9</f>
-        <v/>
-      </c>
-      <c r="W9" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T9="","",U9-J9)</f>
+        <v/>
+      </c>
+      <c r="W9" s="44">
+        <f>IF(T9="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X9" s="57" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -2246,23 +2253,20 @@
           <t>OBS-065</t>
         </is>
       </c>
-      <c r="T10" s="42">
-        <f>I10</f>
-        <v/>
-      </c>
+      <c r="T10" s="42" t="n"/>
       <c r="U10" s="43">
-        <f>T10*N(F10)</f>
+        <f>IF(T10="",0,T10*N(F10))</f>
         <v/>
       </c>
       <c r="V10" s="43">
-        <f>U10-J10</f>
-        <v/>
-      </c>
-      <c r="W10" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T10="","",U10-J10)</f>
+        <v/>
+      </c>
+      <c r="W10" s="44">
+        <f>IF(T10="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X10" s="57" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -2332,23 +2336,20 @@
         </is>
       </c>
       <c r="S11" s="4" t="n"/>
-      <c r="T11" s="42">
-        <f>I11</f>
-        <v/>
-      </c>
+      <c r="T11" s="42" t="n"/>
       <c r="U11" s="43">
-        <f>T11*N(F11)</f>
+        <f>IF(T11="",0,T11*N(F11))</f>
         <v/>
       </c>
       <c r="V11" s="43">
-        <f>U11-J11</f>
-        <v/>
-      </c>
-      <c r="W11" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T11="","",U11-J11)</f>
+        <v/>
+      </c>
+      <c r="W11" s="44">
+        <f>IF(T11="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X11" s="57" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -2422,23 +2423,20 @@
           <t>OBS-042</t>
         </is>
       </c>
-      <c r="T12" s="42">
-        <f>I12</f>
-        <v/>
-      </c>
+      <c r="T12" s="42" t="n"/>
       <c r="U12" s="43">
-        <f>T12*N(F12)</f>
+        <f>IF(T12="",0,T12*N(F12))</f>
         <v/>
       </c>
       <c r="V12" s="43">
-        <f>U12-J12</f>
-        <v/>
-      </c>
-      <c r="W12" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T12="","",U12-J12)</f>
+        <v/>
+      </c>
+      <c r="W12" s="44">
+        <f>IF(T12="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X12" s="57" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -2512,23 +2510,20 @@
           <t>OBS-041</t>
         </is>
       </c>
-      <c r="T13" s="42">
-        <f>I13</f>
-        <v/>
-      </c>
+      <c r="T13" s="42" t="n"/>
       <c r="U13" s="43">
-        <f>T13*N(F13)</f>
+        <f>IF(T13="",0,T13*N(F13))</f>
         <v/>
       </c>
       <c r="V13" s="43">
-        <f>U13-J13</f>
-        <v/>
-      </c>
-      <c r="W13" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T13="","",U13-J13)</f>
+        <v/>
+      </c>
+      <c r="W13" s="44">
+        <f>IF(T13="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X13" s="57" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -2602,23 +2597,20 @@
           <t>OBS-043</t>
         </is>
       </c>
-      <c r="T14" s="42">
-        <f>I14</f>
-        <v/>
-      </c>
+      <c r="T14" s="42" t="n"/>
       <c r="U14" s="43">
-        <f>T14*N(F14)</f>
+        <f>IF(T14="",0,T14*N(F14))</f>
         <v/>
       </c>
       <c r="V14" s="43">
-        <f>U14-J14</f>
-        <v/>
-      </c>
-      <c r="W14" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T14="","",U14-J14)</f>
+        <v/>
+      </c>
+      <c r="W14" s="44">
+        <f>IF(T14="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2692,23 +2684,20 @@
           <t>OBS-053</t>
         </is>
       </c>
-      <c r="T15" s="42">
-        <f>I15</f>
-        <v/>
-      </c>
+      <c r="T15" s="42" t="n"/>
       <c r="U15" s="43">
-        <f>T15*N(F15)</f>
+        <f>IF(T15="",0,T15*N(F15))</f>
         <v/>
       </c>
       <c r="V15" s="43">
-        <f>U15-J15</f>
-        <v/>
-      </c>
-      <c r="W15" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T15="","",U15-J15)</f>
+        <v/>
+      </c>
+      <c r="W15" s="44">
+        <f>IF(T15="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2782,23 +2771,20 @@
           <t>OBS-065</t>
         </is>
       </c>
-      <c r="T16" s="42">
-        <f>I16</f>
-        <v/>
-      </c>
+      <c r="T16" s="42" t="n"/>
       <c r="U16" s="43">
-        <f>T16*N(F16)</f>
+        <f>IF(T16="",0,T16*N(F16))</f>
         <v/>
       </c>
       <c r="V16" s="43">
-        <f>U16-J16</f>
-        <v/>
-      </c>
-      <c r="W16" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T16="","",U16-J16)</f>
+        <v/>
+      </c>
+      <c r="W16" s="44">
+        <f>IF(T16="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X16" s="57" t="n"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -2872,23 +2858,20 @@
           <t>OBS-040</t>
         </is>
       </c>
-      <c r="T17" s="42">
-        <f>I17</f>
-        <v/>
-      </c>
+      <c r="T17" s="42" t="n"/>
       <c r="U17" s="43">
-        <f>T17*N(F17)</f>
+        <f>IF(T17="",0,T17*N(F17))</f>
         <v/>
       </c>
       <c r="V17" s="43">
-        <f>U17-J17</f>
-        <v/>
-      </c>
-      <c r="W17" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T17="","",U17-J17)</f>
+        <v/>
+      </c>
+      <c r="W17" s="44">
+        <f>IF(T17="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X17" s="57" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -2962,23 +2945,20 @@
           <t>OBS-056</t>
         </is>
       </c>
-      <c r="T18" s="42">
-        <f>I18</f>
-        <v/>
-      </c>
+      <c r="T18" s="42" t="n"/>
       <c r="U18" s="43">
-        <f>T18*N(F18)</f>
+        <f>IF(T18="",0,T18*N(F18))</f>
         <v/>
       </c>
       <c r="V18" s="43">
-        <f>U18-J18</f>
-        <v/>
-      </c>
-      <c r="W18" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T18="","",U18-J18)</f>
+        <v/>
+      </c>
+      <c r="W18" s="44">
+        <f>IF(T18="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X18" s="57" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -3052,23 +3032,20 @@
           <t>OBS-056</t>
         </is>
       </c>
-      <c r="T19" s="42">
-        <f>I19</f>
-        <v/>
-      </c>
+      <c r="T19" s="42" t="n"/>
       <c r="U19" s="43">
-        <f>T19*N(F19)</f>
+        <f>IF(T19="",0,T19*N(F19))</f>
         <v/>
       </c>
       <c r="V19" s="43">
-        <f>U19-J19</f>
-        <v/>
-      </c>
-      <c r="W19" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T19="","",U19-J19)</f>
+        <v/>
+      </c>
+      <c r="W19" s="44">
+        <f>IF(T19="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X19" s="57" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -3142,22 +3119,20 @@
           <t>OBS-065</t>
         </is>
       </c>
-      <c r="T20" s="42" t="n">
-        <v>6</v>
-      </c>
+      <c r="T20" s="42" t="n"/>
       <c r="U20" s="43">
-        <f>T20*N(F20)</f>
+        <f>IF(T20="",0,T20*N(F20))</f>
         <v/>
       </c>
       <c r="V20" s="43">
-        <f>U20-J20</f>
-        <v/>
-      </c>
-      <c r="W20" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T20="","",U20-J20)</f>
+        <v/>
+      </c>
+      <c r="W20" s="44">
+        <f>IF(T20="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X20" s="57" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -3231,23 +3206,20 @@
           <t>OBS-064</t>
         </is>
       </c>
-      <c r="T21" s="42">
-        <f>I21</f>
-        <v/>
-      </c>
+      <c r="T21" s="42" t="n"/>
       <c r="U21" s="43">
-        <f>T21*N(F21)</f>
+        <f>IF(T21="",0,T21*N(F21))</f>
         <v/>
       </c>
       <c r="V21" s="43">
-        <f>U21-J21</f>
-        <v/>
-      </c>
-      <c r="W21" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T21="","",U21-J21)</f>
+        <v/>
+      </c>
+      <c r="W21" s="44">
+        <f>IF(T21="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X21" s="57" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -3321,23 +3293,20 @@
           <t>OBS-064</t>
         </is>
       </c>
-      <c r="T22" s="42">
-        <f>I22</f>
-        <v/>
-      </c>
+      <c r="T22" s="42" t="n"/>
       <c r="U22" s="43">
-        <f>T22*N(F22)</f>
+        <f>IF(T22="",0,T22*N(F22))</f>
         <v/>
       </c>
       <c r="V22" s="43">
-        <f>U22-J22</f>
-        <v/>
-      </c>
-      <c r="W22" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T22="","",U22-J22)</f>
+        <v/>
+      </c>
+      <c r="W22" s="44">
+        <f>IF(T22="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X22" s="57" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -3407,23 +3376,20 @@
         </is>
       </c>
       <c r="S23" s="4" t="n"/>
-      <c r="T23" s="42">
-        <f>I23</f>
-        <v/>
-      </c>
+      <c r="T23" s="42" t="n"/>
       <c r="U23" s="43">
-        <f>T23*N(F23)</f>
+        <f>IF(T23="",0,T23*N(F23))</f>
         <v/>
       </c>
       <c r="V23" s="43">
-        <f>U23-J23</f>
-        <v/>
-      </c>
-      <c r="W23" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T23="","",U23-J23)</f>
+        <v/>
+      </c>
+      <c r="W23" s="44">
+        <f>IF(T23="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X23" s="57" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -3493,23 +3459,20 @@
         </is>
       </c>
       <c r="S24" s="4" t="n"/>
-      <c r="T24" s="42">
-        <f>I24</f>
-        <v/>
-      </c>
+      <c r="T24" s="42" t="n"/>
       <c r="U24" s="43">
-        <f>T24*N(F24)</f>
+        <f>IF(T24="",0,T24*N(F24))</f>
         <v/>
       </c>
       <c r="V24" s="43">
-        <f>U24-J24</f>
-        <v/>
-      </c>
-      <c r="W24" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T24="","",U24-J24)</f>
+        <v/>
+      </c>
+      <c r="W24" s="44">
+        <f>IF(T24="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X24" s="57" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -3579,23 +3542,20 @@
         </is>
       </c>
       <c r="S25" s="4" t="n"/>
-      <c r="T25" s="42">
-        <f>I25</f>
-        <v/>
-      </c>
+      <c r="T25" s="42" t="n"/>
       <c r="U25" s="43">
-        <f>T25*N(F25)</f>
+        <f>IF(T25="",0,T25*N(F25))</f>
         <v/>
       </c>
       <c r="V25" s="43">
-        <f>U25-J25</f>
-        <v/>
-      </c>
-      <c r="W25" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T25="","",U25-J25)</f>
+        <v/>
+      </c>
+      <c r="W25" s="44">
+        <f>IF(T25="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X25" s="57" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
@@ -3669,23 +3629,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T26" s="42">
-        <f>I26</f>
-        <v/>
-      </c>
+      <c r="T26" s="42" t="n"/>
       <c r="U26" s="43">
-        <f>T26*N(F26)</f>
+        <f>IF(T26="",0,T26*N(F26))</f>
         <v/>
       </c>
       <c r="V26" s="43">
-        <f>U26-J26</f>
-        <v/>
-      </c>
-      <c r="W26" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T26="","",U26-J26)</f>
+        <v/>
+      </c>
+      <c r="W26" s="44">
+        <f>IF(T26="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3759,23 +3716,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T27" s="42">
-        <f>I27</f>
-        <v/>
-      </c>
+      <c r="T27" s="42" t="n"/>
       <c r="U27" s="43">
-        <f>T27*N(F27)</f>
+        <f>IF(T27="",0,T27*N(F27))</f>
         <v/>
       </c>
       <c r="V27" s="43">
-        <f>U27-J27</f>
-        <v/>
-      </c>
-      <c r="W27" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T27="","",U27-J27)</f>
+        <v/>
+      </c>
+      <c r="W27" s="44">
+        <f>IF(T27="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -3849,23 +3803,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T28" s="42">
-        <f>I28</f>
-        <v/>
-      </c>
+      <c r="T28" s="42" t="n"/>
       <c r="U28" s="43">
-        <f>T28*N(F28)</f>
+        <f>IF(T28="",0,T28*N(F28))</f>
         <v/>
       </c>
       <c r="V28" s="43">
-        <f>U28-J28</f>
-        <v/>
-      </c>
-      <c r="W28" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T28="","",U28-J28)</f>
+        <v/>
+      </c>
+      <c r="W28" s="44">
+        <f>IF(T28="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3939,23 +3890,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T29" s="42">
-        <f>I29</f>
-        <v/>
-      </c>
+      <c r="T29" s="42" t="n"/>
       <c r="U29" s="43">
-        <f>T29*N(F29)</f>
+        <f>IF(T29="",0,T29*N(F29))</f>
         <v/>
       </c>
       <c r="V29" s="43">
-        <f>U29-J29</f>
-        <v/>
-      </c>
-      <c r="W29" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T29="","",U29-J29)</f>
+        <v/>
+      </c>
+      <c r="W29" s="44">
+        <f>IF(T29="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X29" s="57" t="n"/>
     </row>
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
@@ -4029,23 +3977,20 @@
           <t>OBS-049</t>
         </is>
       </c>
-      <c r="T30" s="42">
-        <f>I30</f>
-        <v/>
-      </c>
+      <c r="T30" s="42" t="n"/>
       <c r="U30" s="43">
-        <f>T30*N(F30)</f>
+        <f>IF(T30="",0,T30*N(F30))</f>
         <v/>
       </c>
       <c r="V30" s="43">
-        <f>U30-J30</f>
-        <v/>
-      </c>
-      <c r="W30" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T30="","",U30-J30)</f>
+        <v/>
+      </c>
+      <c r="W30" s="44">
+        <f>IF(T30="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X30" s="57" t="n"/>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -4115,23 +4060,20 @@
         </is>
       </c>
       <c r="S31" s="4" t="n"/>
-      <c r="T31" s="42">
-        <f>I31</f>
-        <v/>
-      </c>
+      <c r="T31" s="42" t="n"/>
       <c r="U31" s="43">
-        <f>T31*N(F31)</f>
+        <f>IF(T31="",0,T31*N(F31))</f>
         <v/>
       </c>
       <c r="V31" s="43">
-        <f>U31-J31</f>
-        <v/>
-      </c>
-      <c r="W31" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T31="","",U31-J31)</f>
+        <v/>
+      </c>
+      <c r="W31" s="44">
+        <f>IF(T31="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X31" s="57" t="n"/>
     </row>
     <row r="32" ht="56" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -4201,23 +4143,20 @@
         </is>
       </c>
       <c r="S32" s="4" t="n"/>
-      <c r="T32" s="42">
-        <f>I32</f>
-        <v/>
-      </c>
+      <c r="T32" s="42" t="n"/>
       <c r="U32" s="43">
-        <f>T32*N(F32)</f>
+        <f>IF(T32="",0,T32*N(F32))</f>
         <v/>
       </c>
       <c r="V32" s="43">
-        <f>U32-J32</f>
-        <v/>
-      </c>
-      <c r="W32" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T32="","",U32-J32)</f>
+        <v/>
+      </c>
+      <c r="W32" s="44">
+        <f>IF(T32="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X32" s="57" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -4303,22 +4242,20 @@
           <t>OBS-016</t>
         </is>
       </c>
-      <c r="T33" s="42" t="n">
-        <v>12</v>
-      </c>
+      <c r="T33" s="42" t="n"/>
       <c r="U33" s="43">
-        <f>T33*N(F33)</f>
+        <f>IF(T33="",0,T33*N(F33))</f>
         <v/>
       </c>
       <c r="V33" s="43">
-        <f>U33-J33</f>
-        <v/>
-      </c>
-      <c r="W33" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T33="","",U33-J33)</f>
+        <v/>
+      </c>
+      <c r="W33" s="44">
+        <f>IF(T33="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X33" s="57" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -4392,23 +4329,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T34" s="42">
-        <f>I34</f>
-        <v/>
-      </c>
+      <c r="T34" s="42" t="n"/>
       <c r="U34" s="43">
-        <f>T34*N(F34)</f>
+        <f>IF(T34="",0,T34*N(F34))</f>
         <v/>
       </c>
       <c r="V34" s="43">
-        <f>U34-J34</f>
-        <v/>
-      </c>
-      <c r="W34" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T34="","",U34-J34)</f>
+        <v/>
+      </c>
+      <c r="W34" s="44">
+        <f>IF(T34="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -4482,23 +4416,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T35" s="42">
-        <f>I35</f>
-        <v/>
-      </c>
+      <c r="T35" s="42" t="n"/>
       <c r="U35" s="43">
-        <f>T35*N(F35)</f>
+        <f>IF(T35="",0,T35*N(F35))</f>
         <v/>
       </c>
       <c r="V35" s="43">
-        <f>U35-J35</f>
-        <v/>
-      </c>
-      <c r="W35" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T35="","",U35-J35)</f>
+        <v/>
+      </c>
+      <c r="W35" s="44">
+        <f>IF(T35="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X35" s="57" t="n"/>
     </row>
     <row r="36" ht="42" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -4572,23 +4503,20 @@
           <t>OBS-053</t>
         </is>
       </c>
-      <c r="T36" s="42">
-        <f>I36</f>
-        <v/>
-      </c>
+      <c r="T36" s="42" t="n"/>
       <c r="U36" s="43">
-        <f>T36*N(F36)</f>
+        <f>IF(T36="",0,T36*N(F36))</f>
         <v/>
       </c>
       <c r="V36" s="43">
-        <f>U36-J36</f>
-        <v/>
-      </c>
-      <c r="W36" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T36="","",U36-J36)</f>
+        <v/>
+      </c>
+      <c r="W36" s="44">
+        <f>IF(T36="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X36" s="57" t="n"/>
     </row>
     <row r="37" ht="56" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -4674,22 +4602,20 @@
           <t>OBS-015</t>
         </is>
       </c>
-      <c r="T37" s="42" t="n">
-        <v>4</v>
-      </c>
+      <c r="T37" s="42" t="n"/>
       <c r="U37" s="43">
-        <f>T37*N(F37)</f>
+        <f>IF(T37="",0,T37*N(F37))</f>
         <v/>
       </c>
       <c r="V37" s="43">
-        <f>U37-J37</f>
-        <v/>
-      </c>
-      <c r="W37" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T37="","",U37-J37)</f>
+        <v/>
+      </c>
+      <c r="W37" s="44">
+        <f>IF(T37="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X37" s="57" t="n"/>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
@@ -4774,23 +4700,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T38" s="42">
-        <f>I38</f>
-        <v/>
-      </c>
+      <c r="T38" s="42" t="n"/>
       <c r="U38" s="43">
-        <f>T38*N(F38)</f>
+        <f>IF(T38="",0,T38*N(F38))</f>
         <v/>
       </c>
       <c r="V38" s="43">
-        <f>U38-J38</f>
-        <v/>
-      </c>
-      <c r="W38" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T38="","",U38-J38)</f>
+        <v/>
+      </c>
+      <c r="W38" s="44">
+        <f>IF(T38="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X38" s="57" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -4875,23 +4798,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T39" s="42">
-        <f>I39</f>
-        <v/>
-      </c>
+      <c r="T39" s="42" t="n"/>
       <c r="U39" s="43">
-        <f>T39*N(F39)</f>
+        <f>IF(T39="",0,T39*N(F39))</f>
         <v/>
       </c>
       <c r="V39" s="43">
-        <f>U39-J39</f>
-        <v/>
-      </c>
-      <c r="W39" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T39="","",U39-J39)</f>
+        <v/>
+      </c>
+      <c r="W39" s="44">
+        <f>IF(T39="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X39" s="57" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -4976,23 +4896,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T40" s="42">
-        <f>I40</f>
-        <v/>
-      </c>
+      <c r="T40" s="42" t="n"/>
       <c r="U40" s="43">
-        <f>T40*N(F40)</f>
+        <f>IF(T40="",0,T40*N(F40))</f>
         <v/>
       </c>
       <c r="V40" s="43">
-        <f>U40-J40</f>
-        <v/>
-      </c>
-      <c r="W40" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T40="","",U40-J40)</f>
+        <v/>
+      </c>
+      <c r="W40" s="44">
+        <f>IF(T40="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X40" s="57" t="n"/>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -5077,23 +4994,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T41" s="42">
-        <f>I41</f>
-        <v/>
-      </c>
+      <c r="T41" s="42" t="n"/>
       <c r="U41" s="43">
-        <f>T41*N(F41)</f>
+        <f>IF(T41="",0,T41*N(F41))</f>
         <v/>
       </c>
       <c r="V41" s="43">
-        <f>U41-J41</f>
-        <v/>
-      </c>
-      <c r="W41" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T41="","",U41-J41)</f>
+        <v/>
+      </c>
+      <c r="W41" s="44">
+        <f>IF(T41="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X41" s="57" t="n"/>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
@@ -5178,23 +5092,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T42" s="42">
-        <f>I42</f>
-        <v/>
-      </c>
+      <c r="T42" s="42" t="n"/>
       <c r="U42" s="43">
-        <f>T42*N(F42)</f>
+        <f>IF(T42="",0,T42*N(F42))</f>
         <v/>
       </c>
       <c r="V42" s="43">
-        <f>U42-J42</f>
-        <v/>
-      </c>
-      <c r="W42" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T42="","",U42-J42)</f>
+        <v/>
+      </c>
+      <c r="W42" s="44">
+        <f>IF(T42="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X42" s="57" t="n"/>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -5279,23 +5190,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T43" s="42">
-        <f>I43</f>
-        <v/>
-      </c>
+      <c r="T43" s="42" t="n"/>
       <c r="U43" s="43">
-        <f>T43*N(F43)</f>
+        <f>IF(T43="",0,T43*N(F43))</f>
         <v/>
       </c>
       <c r="V43" s="43">
-        <f>U43-J43</f>
-        <v/>
-      </c>
-      <c r="W43" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T43="","",U43-J43)</f>
+        <v/>
+      </c>
+      <c r="W43" s="44">
+        <f>IF(T43="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X43" s="57" t="n"/>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -5369,23 +5277,20 @@
           <t>OBS-058</t>
         </is>
       </c>
-      <c r="T44" s="42">
-        <f>I44</f>
-        <v/>
-      </c>
+      <c r="T44" s="42" t="n"/>
       <c r="U44" s="43">
-        <f>T44*N(F44)</f>
+        <f>IF(T44="",0,T44*N(F44))</f>
         <v/>
       </c>
       <c r="V44" s="43">
-        <f>U44-J44</f>
-        <v/>
-      </c>
-      <c r="W44" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T44="","",U44-J44)</f>
+        <v/>
+      </c>
+      <c r="W44" s="44">
+        <f>IF(T44="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X44" s="57" t="n"/>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -5470,23 +5375,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T45" s="42">
-        <f>I45</f>
-        <v/>
-      </c>
+      <c r="T45" s="42" t="n"/>
       <c r="U45" s="43">
-        <f>T45*N(F45)</f>
+        <f>IF(T45="",0,T45*N(F45))</f>
         <v/>
       </c>
       <c r="V45" s="43">
-        <f>U45-J45</f>
-        <v/>
-      </c>
-      <c r="W45" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T45="","",U45-J45)</f>
+        <v/>
+      </c>
+      <c r="W45" s="44">
+        <f>IF(T45="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X45" s="57" t="n"/>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -5571,23 +5473,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T46" s="42">
-        <f>I46</f>
-        <v/>
-      </c>
+      <c r="T46" s="42" t="n"/>
       <c r="U46" s="43">
-        <f>T46*N(F46)</f>
+        <f>IF(T46="",0,T46*N(F46))</f>
         <v/>
       </c>
       <c r="V46" s="43">
-        <f>U46-J46</f>
-        <v/>
-      </c>
-      <c r="W46" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T46="","",U46-J46)</f>
+        <v/>
+      </c>
+      <c r="W46" s="44">
+        <f>IF(T46="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X46" s="57" t="n"/>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -5672,23 +5571,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T47" s="42">
-        <f>I47</f>
-        <v/>
-      </c>
+      <c r="T47" s="42" t="n"/>
       <c r="U47" s="43">
-        <f>T47*N(F47)</f>
+        <f>IF(T47="",0,T47*N(F47))</f>
         <v/>
       </c>
       <c r="V47" s="43">
-        <f>U47-J47</f>
-        <v/>
-      </c>
-      <c r="W47" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T47="","",U47-J47)</f>
+        <v/>
+      </c>
+      <c r="W47" s="44">
+        <f>IF(T47="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X47" s="57" t="n"/>
     </row>
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
@@ -5758,23 +5654,20 @@
         </is>
       </c>
       <c r="S48" s="4" t="n"/>
-      <c r="T48" s="42">
-        <f>I48</f>
-        <v/>
-      </c>
+      <c r="T48" s="42" t="n"/>
       <c r="U48" s="43">
-        <f>T48*N(F48)</f>
+        <f>IF(T48="",0,T48*N(F48))</f>
         <v/>
       </c>
       <c r="V48" s="43">
-        <f>U48-J48</f>
-        <v/>
-      </c>
-      <c r="W48" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T48="","",U48-J48)</f>
+        <v/>
+      </c>
+      <c r="W48" s="44">
+        <f>IF(T48="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X48" s="57" t="n"/>
     </row>
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -5844,23 +5737,20 @@
         </is>
       </c>
       <c r="S49" s="4" t="n"/>
-      <c r="T49" s="42">
-        <f>I49</f>
-        <v/>
-      </c>
+      <c r="T49" s="42" t="n"/>
       <c r="U49" s="43">
-        <f>T49*N(F49)</f>
+        <f>IF(T49="",0,T49*N(F49))</f>
         <v/>
       </c>
       <c r="V49" s="43">
-        <f>U49-J49</f>
-        <v/>
-      </c>
-      <c r="W49" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T49="","",U49-J49)</f>
+        <v/>
+      </c>
+      <c r="W49" s="44">
+        <f>IF(T49="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X49" s="57" t="n"/>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
@@ -5930,23 +5820,20 @@
         </is>
       </c>
       <c r="S50" s="4" t="n"/>
-      <c r="T50" s="42">
-        <f>I50</f>
-        <v/>
-      </c>
+      <c r="T50" s="42" t="n"/>
       <c r="U50" s="43">
-        <f>T50*N(F50)</f>
+        <f>IF(T50="",0,T50*N(F50))</f>
         <v/>
       </c>
       <c r="V50" s="43">
-        <f>U50-J50</f>
-        <v/>
-      </c>
-      <c r="W50" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T50="","",U50-J50)</f>
+        <v/>
+      </c>
+      <c r="W50" s="44">
+        <f>IF(T50="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X50" s="57" t="n"/>
     </row>
     <row r="51" ht="70" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
@@ -6020,23 +5907,20 @@
           <t>OBS-007, OBS-011</t>
         </is>
       </c>
-      <c r="T51" s="42">
-        <f>I51</f>
-        <v/>
-      </c>
+      <c r="T51" s="42" t="n"/>
       <c r="U51" s="43">
-        <f>T51*N(F51)</f>
+        <f>IF(T51="",0,T51*N(F51))</f>
         <v/>
       </c>
       <c r="V51" s="43">
-        <f>U51-J51</f>
-        <v/>
-      </c>
-      <c r="W51" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T51="","",U51-J51)</f>
+        <v/>
+      </c>
+      <c r="W51" s="44">
+        <f>IF(T51="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X51" s="57" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -6122,22 +6006,20 @@
           <t>OBS-014</t>
         </is>
       </c>
-      <c r="T52" s="42" t="n">
-        <v>4</v>
-      </c>
+      <c r="T52" s="42" t="n"/>
       <c r="U52" s="43">
-        <f>T52*N(F52)</f>
+        <f>IF(T52="",0,T52*N(F52))</f>
         <v/>
       </c>
       <c r="V52" s="43">
-        <f>U52-J52</f>
-        <v/>
-      </c>
-      <c r="W52" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T52="","",U52-J52)</f>
+        <v/>
+      </c>
+      <c r="W52" s="44">
+        <f>IF(T52="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X52" s="57" t="n"/>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -6207,23 +6089,20 @@
         </is>
       </c>
       <c r="S53" s="4" t="n"/>
-      <c r="T53" s="42">
-        <f>I53</f>
-        <v/>
-      </c>
+      <c r="T53" s="42" t="n"/>
       <c r="U53" s="43">
-        <f>T53*N(F53)</f>
+        <f>IF(T53="",0,T53*N(F53))</f>
         <v/>
       </c>
       <c r="V53" s="43">
-        <f>U53-J53</f>
-        <v/>
-      </c>
-      <c r="W53" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T53="","",U53-J53)</f>
+        <v/>
+      </c>
+      <c r="W53" s="44">
+        <f>IF(T53="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X53" s="57" t="n"/>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
@@ -6293,23 +6172,20 @@
         </is>
       </c>
       <c r="S54" s="4" t="n"/>
-      <c r="T54" s="42">
-        <f>I54</f>
-        <v/>
-      </c>
+      <c r="T54" s="42" t="n"/>
       <c r="U54" s="43">
-        <f>T54*N(F54)</f>
+        <f>IF(T54="",0,T54*N(F54))</f>
         <v/>
       </c>
       <c r="V54" s="43">
-        <f>U54-J54</f>
-        <v/>
-      </c>
-      <c r="W54" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T54="","",U54-J54)</f>
+        <v/>
+      </c>
+      <c r="W54" s="44">
+        <f>IF(T54="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X54" s="57" t="n"/>
     </row>
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
@@ -6383,22 +6259,20 @@
           <t>OBS-009</t>
         </is>
       </c>
-      <c r="T55" s="42" t="n">
-        <v>4</v>
-      </c>
+      <c r="T55" s="42" t="n"/>
       <c r="U55" s="43">
-        <f>T55*N(F55)</f>
+        <f>IF(T55="",0,T55*N(F55))</f>
         <v/>
       </c>
       <c r="V55" s="43">
-        <f>U55-J55</f>
-        <v/>
-      </c>
-      <c r="W55" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T55="","",U55-J55)</f>
+        <v/>
+      </c>
+      <c r="W55" s="44">
+        <f>IF(T55="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X55" s="57" t="n"/>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -6472,23 +6346,20 @@
           <t>OBS-057</t>
         </is>
       </c>
-      <c r="T56" s="42">
-        <f>I56</f>
-        <v/>
-      </c>
+      <c r="T56" s="42" t="n"/>
       <c r="U56" s="43">
-        <f>T56*N(F56)</f>
+        <f>IF(T56="",0,T56*N(F56))</f>
         <v/>
       </c>
       <c r="V56" s="43">
-        <f>U56-J56</f>
-        <v/>
-      </c>
-      <c r="W56" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T56="","",U56-J56)</f>
+        <v/>
+      </c>
+      <c r="W56" s="44">
+        <f>IF(T56="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X56" s="57" t="n"/>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -6562,23 +6433,20 @@
           <t>OBS-051</t>
         </is>
       </c>
-      <c r="T57" s="42">
-        <f>I57</f>
-        <v/>
-      </c>
+      <c r="T57" s="42" t="n"/>
       <c r="U57" s="43">
-        <f>T57*N(F57)</f>
+        <f>IF(T57="",0,T57*N(F57))</f>
         <v/>
       </c>
       <c r="V57" s="43">
-        <f>U57-J57</f>
-        <v/>
-      </c>
-      <c r="W57" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T57="","",U57-J57)</f>
+        <v/>
+      </c>
+      <c r="W57" s="44">
+        <f>IF(T57="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X57" s="57" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
@@ -6663,23 +6531,20 @@
           <t>OBS-060</t>
         </is>
       </c>
-      <c r="T58" s="42">
-        <f>I58</f>
-        <v/>
-      </c>
+      <c r="T58" s="42" t="n"/>
       <c r="U58" s="43">
-        <f>T58*N(F58)</f>
+        <f>IF(T58="",0,T58*N(F58))</f>
         <v/>
       </c>
       <c r="V58" s="43">
-        <f>U58-J58</f>
-        <v/>
-      </c>
-      <c r="W58" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T58="","",U58-J58)</f>
+        <v/>
+      </c>
+      <c r="W58" s="44">
+        <f>IF(T58="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X58" s="57" t="n"/>
     </row>
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -6753,23 +6618,20 @@
           <t>OBS-060</t>
         </is>
       </c>
-      <c r="T59" s="42">
-        <f>I59</f>
-        <v/>
-      </c>
+      <c r="T59" s="42" t="n"/>
       <c r="U59" s="43">
-        <f>T59*N(F59)</f>
+        <f>IF(T59="",0,T59*N(F59))</f>
         <v/>
       </c>
       <c r="V59" s="43">
-        <f>U59-J59</f>
-        <v/>
-      </c>
-      <c r="W59" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T59="","",U59-J59)</f>
+        <v/>
+      </c>
+      <c r="W59" s="44">
+        <f>IF(T59="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X59" s="57" t="n"/>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -6843,23 +6705,20 @@
           <t>OBS-060</t>
         </is>
       </c>
-      <c r="T60" s="42">
-        <f>I60</f>
-        <v/>
-      </c>
+      <c r="T60" s="42" t="n"/>
       <c r="U60" s="43">
-        <f>T60*N(F60)</f>
+        <f>IF(T60="",0,T60*N(F60))</f>
         <v/>
       </c>
       <c r="V60" s="43">
-        <f>U60-J60</f>
-        <v/>
-      </c>
-      <c r="W60" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T60="","",U60-J60)</f>
+        <v/>
+      </c>
+      <c r="W60" s="44">
+        <f>IF(T60="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X60" s="57" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="21" t="n"/>
@@ -6996,23 +6855,20 @@
           <t>OBS-038, OBS-064</t>
         </is>
       </c>
-      <c r="T63" s="42">
-        <f>I63</f>
-        <v/>
-      </c>
+      <c r="T63" s="42" t="n"/>
       <c r="U63" s="43">
-        <f>T63*N(F63)</f>
+        <f>IF(T63="",0,T63*N(F63))</f>
         <v/>
       </c>
       <c r="V63" s="43">
-        <f>U63-J63</f>
-        <v/>
-      </c>
-      <c r="W63" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T63="","",U63-J63)</f>
+        <v/>
+      </c>
+      <c r="W63" s="44">
+        <f>IF(T63="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X63" s="57" t="n"/>
     </row>
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
@@ -7077,23 +6933,20 @@
           <t>OBS-056, OBS-064</t>
         </is>
       </c>
-      <c r="T64" s="42">
-        <f>I64</f>
-        <v/>
-      </c>
+      <c r="T64" s="42" t="n"/>
       <c r="U64" s="43">
-        <f>T64*N(F64)</f>
+        <f>IF(T64="",0,T64*N(F64))</f>
         <v/>
       </c>
       <c r="V64" s="43">
-        <f>U64-J64</f>
-        <v/>
-      </c>
-      <c r="W64" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T64="","",U64-J64)</f>
+        <v/>
+      </c>
+      <c r="W64" s="44">
+        <f>IF(T64="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X64" s="57" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -7158,23 +7011,20 @@
           <t>OBS-064</t>
         </is>
       </c>
-      <c r="T65" s="42">
-        <f>I65</f>
-        <v/>
-      </c>
+      <c r="T65" s="42" t="n"/>
       <c r="U65" s="43">
-        <f>T65*N(F65)</f>
+        <f>IF(T65="",0,T65*N(F65))</f>
         <v/>
       </c>
       <c r="V65" s="43">
-        <f>U65-J65</f>
-        <v/>
-      </c>
-      <c r="W65" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T65="","",U65-J65)</f>
+        <v/>
+      </c>
+      <c r="W65" s="44">
+        <f>IF(T65="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X65" s="57" t="n"/>
     </row>
     <row r="66" ht="42" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
@@ -7251,23 +7101,20 @@
           <t>OBS-050, OBS-038</t>
         </is>
       </c>
-      <c r="T66" s="42">
-        <f>I66</f>
-        <v/>
-      </c>
+      <c r="T66" s="42" t="n"/>
       <c r="U66" s="43">
-        <f>T66*N(F66)</f>
+        <f>IF(T66="",0,T66*N(F66))</f>
         <v/>
       </c>
       <c r="V66" s="43">
-        <f>U66-J66</f>
-        <v/>
-      </c>
-      <c r="W66" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T66="","",U66-J66)</f>
+        <v/>
+      </c>
+      <c r="W66" s="44">
+        <f>IF(T66="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X66" s="57" t="n"/>
     </row>
     <row r="67" ht="42" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -7344,23 +7191,20 @@
           <t>OBS-046, OBS-038</t>
         </is>
       </c>
-      <c r="T67" s="42">
-        <f>I67</f>
-        <v/>
-      </c>
+      <c r="T67" s="42" t="n"/>
       <c r="U67" s="43">
-        <f>T67*N(F67)</f>
+        <f>IF(T67="",0,T67*N(F67))</f>
         <v/>
       </c>
       <c r="V67" s="43">
-        <f>U67-J67</f>
-        <v/>
-      </c>
-      <c r="W67" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T67="","",U67-J67)</f>
+        <v/>
+      </c>
+      <c r="W67" s="44">
+        <f>IF(T67="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X67" s="57" t="n"/>
     </row>
     <row r="68" ht="42" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
@@ -7437,23 +7281,20 @@
           <t>OBS-047, OBS-038</t>
         </is>
       </c>
-      <c r="T68" s="42">
-        <f>I68</f>
-        <v/>
-      </c>
+      <c r="T68" s="42" t="n"/>
       <c r="U68" s="43">
-        <f>T68*N(F68)</f>
+        <f>IF(T68="",0,T68*N(F68))</f>
         <v/>
       </c>
       <c r="V68" s="43">
-        <f>U68-J68</f>
-        <v/>
-      </c>
-      <c r="W68" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T68="","",U68-J68)</f>
+        <v/>
+      </c>
+      <c r="W68" s="44">
+        <f>IF(T68="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X68" s="57" t="n"/>
     </row>
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -7530,23 +7371,20 @@
           <t>OBS-037, OBS-032</t>
         </is>
       </c>
-      <c r="T69" s="42">
-        <f>I69</f>
-        <v/>
-      </c>
+      <c r="T69" s="42" t="n"/>
       <c r="U69" s="43">
-        <f>T69*N(F69)</f>
+        <f>IF(T69="",0,T69*N(F69))</f>
         <v/>
       </c>
       <c r="V69" s="43">
-        <f>U69-J69</f>
-        <v/>
-      </c>
-      <c r="W69" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T69="","",U69-J69)</f>
+        <v/>
+      </c>
+      <c r="W69" s="44">
+        <f>IF(T69="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X69" s="57" t="n"/>
     </row>
     <row r="70" ht="42" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
@@ -7623,23 +7461,20 @@
           <t>OBS-036, OBS-028, OBS-029</t>
         </is>
       </c>
-      <c r="T70" s="42">
-        <f>I70</f>
-        <v/>
-      </c>
+      <c r="T70" s="42" t="n"/>
       <c r="U70" s="43">
-        <f>T70*N(F70)</f>
+        <f>IF(T70="",0,T70*N(F70))</f>
         <v/>
       </c>
       <c r="V70" s="43">
-        <f>U70-J70</f>
-        <v/>
-      </c>
-      <c r="W70" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T70="","",U70-J70)</f>
+        <v/>
+      </c>
+      <c r="W70" s="44">
+        <f>IF(T70="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X70" s="57" t="n"/>
     </row>
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -7704,23 +7539,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T71" s="42">
-        <f>I71</f>
-        <v/>
-      </c>
+      <c r="T71" s="42" t="n"/>
       <c r="U71" s="43">
-        <f>T71*N(F71)</f>
+        <f>IF(T71="",0,T71*N(F71))</f>
         <v/>
       </c>
       <c r="V71" s="43">
-        <f>U71-J71</f>
-        <v/>
-      </c>
-      <c r="W71" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T71="","",U71-J71)</f>
+        <v/>
+      </c>
+      <c r="W71" s="44">
+        <f>IF(T71="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X71" s="57" t="n"/>
     </row>
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
@@ -7785,23 +7617,20 @@
           <t>OBS-006</t>
         </is>
       </c>
-      <c r="T72" s="42">
-        <f>I72</f>
-        <v/>
-      </c>
+      <c r="T72" s="42" t="n"/>
       <c r="U72" s="43">
-        <f>T72*N(F72)</f>
+        <f>IF(T72="",0,T72*N(F72))</f>
         <v/>
       </c>
       <c r="V72" s="43">
-        <f>U72-J72</f>
-        <v/>
-      </c>
-      <c r="W72" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T72="","",U72-J72)</f>
+        <v/>
+      </c>
+      <c r="W72" s="44">
+        <f>IF(T72="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X72" s="57" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -7877,23 +7706,20 @@
           <t>OBS-049</t>
         </is>
       </c>
-      <c r="T73" s="42">
-        <f>I73</f>
-        <v/>
-      </c>
+      <c r="T73" s="42" t="n"/>
       <c r="U73" s="43">
-        <f>T73*N(F73)</f>
+        <f>IF(T73="",0,T73*N(F73))</f>
         <v/>
       </c>
       <c r="V73" s="43">
-        <f>U73-J73</f>
-        <v/>
-      </c>
-      <c r="W73" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T73="","",U73-J73)</f>
+        <v/>
+      </c>
+      <c r="W73" s="44">
+        <f>IF(T73="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X73" s="57" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -7969,23 +7795,20 @@
           <t>OBS-049</t>
         </is>
       </c>
-      <c r="T74" s="42">
-        <f>I74</f>
-        <v/>
-      </c>
+      <c r="T74" s="42" t="n"/>
       <c r="U74" s="43">
-        <f>T74*N(F74)</f>
+        <f>IF(T74="",0,T74*N(F74))</f>
         <v/>
       </c>
       <c r="V74" s="43">
-        <f>U74-J74</f>
-        <v/>
-      </c>
-      <c r="W74" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T74="","",U74-J74)</f>
+        <v/>
+      </c>
+      <c r="W74" s="44">
+        <f>IF(T74="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X74" s="57" t="n"/>
     </row>
     <row r="75" ht="98" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
@@ -8050,23 +7873,20 @@
           <t>OBS-053</t>
         </is>
       </c>
-      <c r="T75" s="42">
-        <f>I75</f>
-        <v/>
-      </c>
+      <c r="T75" s="42" t="n"/>
       <c r="U75" s="43">
-        <f>T75*N(F75)</f>
+        <f>IF(T75="",0,T75*N(F75))</f>
         <v/>
       </c>
       <c r="V75" s="43">
-        <f>U75-J75</f>
-        <v/>
-      </c>
-      <c r="W75" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T75="","",U75-J75)</f>
+        <v/>
+      </c>
+      <c r="W75" s="44">
+        <f>IF(T75="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X75" s="57" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
@@ -8142,23 +7962,20 @@
           <t>OBS-059</t>
         </is>
       </c>
-      <c r="T76" s="42">
-        <f>I76</f>
-        <v/>
-      </c>
+      <c r="T76" s="42" t="n"/>
       <c r="U76" s="43">
-        <f>T76*N(F76)</f>
+        <f>IF(T76="",0,T76*N(F76))</f>
         <v/>
       </c>
       <c r="V76" s="43">
-        <f>U76-J76</f>
-        <v/>
-      </c>
-      <c r="W76" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T76="","",U76-J76)</f>
+        <v/>
+      </c>
+      <c r="W76" s="44">
+        <f>IF(T76="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X76" s="57" t="n"/>
     </row>
     <row r="77" ht="42" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
@@ -8235,23 +8052,20 @@
           <t>OBS-007, OBS-008</t>
         </is>
       </c>
-      <c r="T77" s="42">
-        <f>I77</f>
-        <v/>
-      </c>
+      <c r="T77" s="42" t="n"/>
       <c r="U77" s="43">
-        <f>T77*N(F77)</f>
+        <f>IF(T77="",0,T77*N(F77))</f>
         <v/>
       </c>
       <c r="V77" s="43">
-        <f>U77-J77</f>
-        <v/>
-      </c>
-      <c r="W77" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T77="","",U77-J77)</f>
+        <v/>
+      </c>
+      <c r="W77" s="44">
+        <f>IF(T77="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X77" s="57" t="n"/>
     </row>
     <row r="78" ht="42" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
@@ -8328,22 +8142,20 @@
           <t>OBS-011, OBS-013</t>
         </is>
       </c>
-      <c r="T78" s="42" t="n">
-        <v>6</v>
-      </c>
+      <c r="T78" s="42" t="n"/>
       <c r="U78" s="43">
-        <f>T78*N(F78)</f>
+        <f>IF(T78="",0,T78*N(F78))</f>
         <v/>
       </c>
       <c r="V78" s="43">
-        <f>U78-J78</f>
-        <v/>
-      </c>
-      <c r="W78" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T78="","",U78-J78)</f>
+        <v/>
+      </c>
+      <c r="W78" s="44">
+        <f>IF(T78="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X78" s="57" t="n"/>
     </row>
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
@@ -8420,23 +8232,20 @@
           <t>OBS-017</t>
         </is>
       </c>
-      <c r="T79" s="42">
-        <f>I79</f>
-        <v/>
-      </c>
+      <c r="T79" s="42" t="n"/>
       <c r="U79" s="43">
-        <f>T79*N(F79)</f>
+        <f>IF(T79="",0,T79*N(F79))</f>
         <v/>
       </c>
       <c r="V79" s="43">
-        <f>U79-J79</f>
-        <v/>
-      </c>
-      <c r="W79" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T79="","",U79-J79)</f>
+        <v/>
+      </c>
+      <c r="W79" s="44">
+        <f>IF(T79="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X79" s="57" t="n"/>
     </row>
     <row r="80" ht="56" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
@@ -8513,22 +8322,20 @@
           <t>OBS-012, OBS-013</t>
         </is>
       </c>
-      <c r="T80" s="42" t="n">
-        <v>0</v>
-      </c>
+      <c r="T80" s="42" t="n"/>
       <c r="U80" s="43">
-        <f>T80*N(F80)</f>
+        <f>IF(T80="",0,T80*N(F80))</f>
         <v/>
       </c>
       <c r="V80" s="43">
-        <f>U80-J80</f>
-        <v/>
-      </c>
-      <c r="W80" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T80="","",U80-J80)</f>
+        <v/>
+      </c>
+      <c r="W80" s="44">
+        <f>IF(T80="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X80" s="57" t="n"/>
     </row>
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
@@ -8605,22 +8412,20 @@
           <t>OBS-009, OBS-010</t>
         </is>
       </c>
-      <c r="T81" s="42" t="n">
-        <v>0</v>
-      </c>
+      <c r="T81" s="42" t="n"/>
       <c r="U81" s="43">
-        <f>T81*N(F81)</f>
+        <f>IF(T81="",0,T81*N(F81))</f>
         <v/>
       </c>
       <c r="V81" s="43">
-        <f>U81-J81</f>
-        <v/>
-      </c>
-      <c r="W81" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T81="","",U81-J81)</f>
+        <v/>
+      </c>
+      <c r="W81" s="44">
+        <f>IF(T81="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X81" s="57" t="n"/>
     </row>
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
@@ -8697,23 +8502,20 @@
           <t>OBS-017</t>
         </is>
       </c>
-      <c r="T82" s="42">
-        <f>I82</f>
-        <v/>
-      </c>
+      <c r="T82" s="42" t="n"/>
       <c r="U82" s="43">
-        <f>T82*N(F82)</f>
+        <f>IF(T82="",0,T82*N(F82))</f>
         <v/>
       </c>
       <c r="V82" s="43">
-        <f>U82-J82</f>
-        <v/>
-      </c>
-      <c r="W82" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T82="","",U82-J82)</f>
+        <v/>
+      </c>
+      <c r="W82" s="44">
+        <f>IF(T82="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X82" s="57" t="n"/>
     </row>
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -8778,23 +8580,20 @@
           <t>OBS-051</t>
         </is>
       </c>
-      <c r="T83" s="42">
-        <f>I83</f>
-        <v/>
-      </c>
+      <c r="T83" s="42" t="n"/>
       <c r="U83" s="43">
-        <f>T83*N(F83)</f>
+        <f>IF(T83="",0,T83*N(F83))</f>
         <v/>
       </c>
       <c r="V83" s="43">
-        <f>U83-J83</f>
-        <v/>
-      </c>
-      <c r="W83" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T83="","",U83-J83)</f>
+        <v/>
+      </c>
+      <c r="W83" s="44">
+        <f>IF(T83="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X83" s="57" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="21" t="n"/>
@@ -8931,23 +8730,20 @@
           <t>OBS-061</t>
         </is>
       </c>
-      <c r="T86" s="42">
-        <f>I86</f>
-        <v/>
-      </c>
+      <c r="T86" s="42" t="n"/>
       <c r="U86" s="43">
-        <f>T86*N(F86)</f>
+        <f>IF(T86="",0,T86*N(F86))</f>
         <v/>
       </c>
       <c r="V86" s="43">
-        <f>U86-J86</f>
-        <v/>
-      </c>
-      <c r="W86" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T86="","",U86-J86)</f>
+        <v/>
+      </c>
+      <c r="W86" s="44">
+        <f>IF(T86="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X86" s="57" t="n"/>
     </row>
     <row r="87" ht="56" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -9012,23 +8808,20 @@
           <t>OBS-061, OBS-001</t>
         </is>
       </c>
-      <c r="T87" s="42">
-        <f>I87</f>
-        <v/>
-      </c>
+      <c r="T87" s="42" t="n"/>
       <c r="U87" s="43">
-        <f>T87*N(F87)</f>
+        <f>IF(T87="",0,T87*N(F87))</f>
         <v/>
       </c>
       <c r="V87" s="43">
-        <f>U87-J87</f>
-        <v/>
-      </c>
-      <c r="W87" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T87="","",U87-J87)</f>
+        <v/>
+      </c>
+      <c r="W87" s="44">
+        <f>IF(T87="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X87" s="57" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
@@ -9093,22 +8886,20 @@
           <t>OBS-062</t>
         </is>
       </c>
-      <c r="T88" s="42" t="n">
-        <v>0</v>
-      </c>
+      <c r="T88" s="42" t="n"/>
       <c r="U88" s="43">
-        <f>T88*N(F88)</f>
+        <f>IF(T88="",0,T88*N(F88))</f>
         <v/>
       </c>
       <c r="V88" s="43">
-        <f>U88-J88</f>
-        <v/>
-      </c>
-      <c r="W88" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T88="","",U88-J88)</f>
+        <v/>
+      </c>
+      <c r="W88" s="44">
+        <f>IF(T88="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X88" s="57" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="21" t="n"/>
@@ -9253,23 +9044,20 @@
           <t>OBS-040</t>
         </is>
       </c>
-      <c r="T91" s="42">
-        <f>I91</f>
-        <v/>
-      </c>
+      <c r="T91" s="42" t="n"/>
       <c r="U91" s="43">
-        <f>T91*N(F91)</f>
+        <f>IF(T91="",0,T91*N(F91))</f>
         <v/>
       </c>
       <c r="V91" s="43">
-        <f>U91</f>
-        <v/>
-      </c>
-      <c r="W91" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T91="","",U91)</f>
+        <v/>
+      </c>
+      <c r="W91" s="44">
+        <f>IF(T91="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X91" s="57" t="n"/>
     </row>
     <row r="92" ht="28" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -9340,22 +9128,20 @@
           <t>OBS-063</t>
         </is>
       </c>
-      <c r="T92" s="42" t="n">
-        <v>1</v>
-      </c>
+      <c r="T92" s="42" t="n"/>
       <c r="U92" s="43">
-        <f>T92*N(F92)</f>
+        <f>IF(T92="",0,T92*N(F92))</f>
         <v/>
       </c>
       <c r="V92" s="43">
-        <f>U92</f>
-        <v/>
-      </c>
-      <c r="W92" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+        <f>IF(T92="","",U92)</f>
+        <v/>
+      </c>
+      <c r="W92" s="44">
+        <f>IF(T92="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X92" s="57" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -9428,23 +9214,20 @@
           <t>OBS-063</t>
         </is>
       </c>
-      <c r="T93" s="42">
-        <f>I93</f>
-        <v/>
-      </c>
+      <c r="T93" s="42" t="n"/>
       <c r="U93" s="43">
-        <f>T93*N(F93)</f>
+        <f>IF(T93="",0,T93*N(F93))</f>
         <v/>
       </c>
       <c r="V93" s="43">
-        <f>U93</f>
-        <v/>
-      </c>
-      <c r="W93" s="44" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
+        <f>IF(T93="","",U93)</f>
+        <v/>
+      </c>
+      <c r="W93" s="44">
+        <f>IF(T93="","Pendiente","Validada")</f>
+        <v/>
+      </c>
+      <c r="X93" s="57" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="21" t="n"/>
@@ -9493,7 +9276,6 @@
       </c>
       <c r="W94" s="46" t="n"/>
     </row>
-    <row r="95"/>
     <row r="96">
       <c r="C96" s="10" t="inlineStr">
         <is>
@@ -9527,7 +9309,6 @@
         <v/>
       </c>
     </row>
-    <row r="99"/>
     <row r="100">
       <c r="C100" s="13" t="inlineStr">
         <is>
@@ -9538,96 +9319,110 @@
     <row r="102">
       <c r="C102" s="51" t="inlineStr">
         <is>
-          <t>BALANCE AJUSTADO (cantidades validadas por el supervisor)</t>
+          <t>PRESUPUESTO CON CANTIDADES VALIDADAS POR EL SUPERVISOR</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="C103" s="52" t="inlineStr">
         <is>
-          <t>VALOR DEL ACTA – ítems eléctricos (Cap. 1 + Cap. 4 + IN14)</t>
+          <t>Ítems eléctricos validados (Cap. 1 + Cap. 4 + IN14)</t>
         </is>
       </c>
       <c r="U103" s="47">
-        <f>J7+J61+J84</f>
+        <f>U7+U61+U84</f>
         <v/>
       </c>
     </row>
     <row r="104">
       <c r="C104" s="52" t="inlineStr">
         <is>
-          <t>VALOR BALANCE AJUSTADO – ítems eléctricos (Cap. 1 + Cap. 4 + IN14)</t>
+          <t>Ítems nuevos necesarios validados</t>
         </is>
       </c>
       <c r="U104" s="47">
-        <f>U7+U61+U84</f>
+        <f>U94</f>
         <v/>
       </c>
     </row>
     <row r="105">
       <c r="C105" s="52" t="inlineStr">
         <is>
-          <t>Ítems nuevos necesarios (transformador, postes de fibra, certificación)</t>
+          <t>Otros ítems relacionados validados</t>
         </is>
       </c>
       <c r="U105" s="47">
-        <f>U94</f>
+        <f>U89</f>
         <v/>
       </c>
     </row>
     <row r="106">
       <c r="C106" s="52" t="inlineStr">
         <is>
-          <t>Otros ítems relacionados (trámites, ajuste de estudios, instalaciones internas)</t>
+          <t>PRESUPUESTO TOTAL VALIDADO</t>
         </is>
       </c>
       <c r="U106" s="47">
-        <f>U89</f>
+        <f>U103+U104+U105</f>
         <v/>
       </c>
     </row>
     <row r="107">
       <c r="C107" s="52" t="inlineStr">
         <is>
-          <t>TOTAL BALANCE AJUSTADO</t>
+          <t>Referencia: valor del acta (Cap. 1 + Cap. 4 + IN14 + otros)</t>
         </is>
       </c>
       <c r="U107" s="47">
-        <f>U104+U105+U106</f>
+        <f>J7+J61+J84+J89</f>
         <v/>
       </c>
     </row>
     <row r="108">
       <c r="C108" s="52" t="inlineStr">
         <is>
-          <t>Diferencia frente al acta (ajustado − acta)</t>
+          <t>Diferencia (presupuesto validado − acta)</t>
         </is>
       </c>
       <c r="U108" s="47">
-        <f>U107-U103</f>
+        <f>U106-U107</f>
         <v/>
       </c>
     </row>
     <row r="109">
       <c r="C109" s="52" t="inlineStr">
         <is>
-          <t>De este total, valor aún PENDIENTE de validar</t>
-        </is>
-      </c>
-      <c r="U109" s="47">
-        <f>SUMIF(W5:W100,"Pendiente",U5:U100)-U7*0</f>
+          <t>Ítems pendientes de validar (cantidad)</t>
+        </is>
+      </c>
+      <c r="U109" s="58">
+        <f>COUNTIF(W5:W99,"Pendiente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="C110" s="52" t="inlineStr">
+        <is>
+          <t>Valor del acta de los ítems pendientes de validar</t>
+        </is>
+      </c>
+      <c r="U110" s="47">
+        <f>SUMIFS(J5:J100,W5:W100,"Pendiente",B5:B100,"&lt;&gt;Nuevo")</f>
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="C111" s="53" t="inlineStr">
-        <is>
-          <t>Cantidad ajustada = decisión del supervisor (Validada) o cantidad del acta mientras no se valide (Pendiente). Celdas amarillas editables: al cambiar una cantidad, todos los totales se recalculan. Ítems retirados y los que concuerdan con los documentos se marcan Validada.</t>
+      <c r="C111" s="53" t="n"/>
+    </row>
+    <row r="112">
+      <c r="C112" s="53" t="inlineStr">
+        <is>
+          <t>Diligenciar la columna T con la cantidad validada de cada ítem (0 si se retira). El presupuesto suma únicamente lo diligenciado; los ítems en blanco figuran como Pendiente y no suman.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:W100"/>
+  <autoFilter ref="A4:X99"/>
   <conditionalFormatting sqref="O5:O95">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Concuerda"</formula>
@@ -9656,10 +9451,7 @@
       <formula>"Pendiente"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="W5:W100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Validada,Pendiente"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="O5:O100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$F$2:$F$7</formula1>
     </dataValidation>

</xml_diff>